<commit_message>
Add Rpt_Start/End_Dt_Key + Run_Ty to CRC, one-active-anchor-per-grouping governance, extended anchor-switch example
</commit_message>
<xml_diff>
--- a/mock-data/cms_compliance_framework_tables.xlsx
+++ b/mock-data/cms_compliance_framework_tables.xlsx
@@ -18,10 +18,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ComplianceSourceSystem'!$A$1:$D$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ComplianceRunType'!$A$1:$C$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ComplianceRunType'!$A$1:$C$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ComplianceDataSetSourceXwalk'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ComplianceRequestControl'!$A$1:$M$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ComplianceBatchOverride'!$A$1:$M$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ComplianceRequestControl'!$A$1:$P$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ComplianceBatchOverride'!$A$1:$T$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ComplianceExtractControl'!$A$1:$M$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'CMS_ComplianceExceptionsAudit'!$A$1:$H$7</definedName>
   </definedNames>
@@ -51,7 +51,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +82,12 @@
         <bgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+        <bgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -109,7 +115,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -121,6 +127,7 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -490,7 +497,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -534,11 +541,11 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Run type master (schema reference)</t>
+          <t>Run type master - CMS (fixed reporting period) and DAILY (single day) used in the examples</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +556,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Carry-forward eligibility + config, per source (schema reference)</t>
+          <t>Carry-forward eligibility + config, per source/run type (schema reference)</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -564,11 +571,11 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CRC - one row per source/table/date, current-state, updated in place</t>
+          <t>CRC - one row per source/table/run type/date, current-state, updated in place</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -579,11 +586,11 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Sparse gate for reuse + reopen - carry-forward, late arrival, correction, all in one table via Override_Ty</t>
+          <t>Sparse gate for reuse + reopen - one APPROVED row max per project/table/source/run type/reporting period</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -758,11 +765,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -786,20 +793,35 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>DAILY</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Daily submission cadence</t>
+          <t>Fixed CMS program-audit reporting period, daily runs within it</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
         <v>1</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Single business day per run, prior-day cadence</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C2"/>
+  <autoFilter ref="A1:C3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -871,7 +893,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>DAILY</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -993,22 +1015,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="19" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1034,45 +1059,60 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
+          <t>Run_Ty</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
           <t>Req_Dt_Key</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Rpt_Start_Dt_Key</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Rpt_End_Dt_Key</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Btch_ID</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Req_Stat</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>File_Received_Ind</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Resolution_Ty</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Used_Btch_ID</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Late_Arrival_Ind</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Batch_Close_Ind</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Batch_Closed_By</t>
         </is>
@@ -1099,45 +1139,60 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_DAILY_2026_1</t>
-        </is>
-      </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
           <t>RULES_PASSED</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1164,41 +1219,56 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
           <t>2026-01-02</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>20260102_PROGAUDIT_ODAG1_2001_DAILY_2026_1</t>
-        </is>
-      </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
           <t>DATA_NOT_PROVIDED</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="J3" s="5" t="n"/>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="M3" s="5" t="n"/>
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1225,301 +1295,380 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
           <t>2026-01-03</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>20260103_PROGAUDIT_ODAG1_2001_DAILY_2026_1</t>
-        </is>
-      </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>20260103_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
           <t>EXTRACTED</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
+      <c r="L4" s="6" t="inlineStr">
         <is>
           <t>CARRIED_FORWARD</t>
         </is>
       </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="M4" s="6" t="inlineStr">
+        <is>
+          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
+      <c r="O4" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="P4" s="6" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>PROGAUDIT</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>2001</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>2026-01-04</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>20260104_PROGAUDIT_ODAG1_2001_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>RULES_PASSED</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>PROGAUDIT</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>ODAG1</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>20260105_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>EXTRACTED</t>
         </is>
       </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>CARRIED_FORWARD</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="M6" s="6" t="inlineStr">
+        <is>
+          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
+      <c r="O6" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="P6" s="6" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>PROGAUDIT</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>2001</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr">
+        <is>
+          <t>EXTRACTED</t>
+        </is>
+      </c>
+      <c r="K7" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>CARRIED_FORWARD</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="inlineStr">
+        <is>
+          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="N7" s="7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O7" s="7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P7" s="7" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>PARTCODR</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ROPENS</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>1001</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>20260105_PROGAUDIT_ODAG1_2001_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>DATA_NOT_PROVIDED</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACTED</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="n"/>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M6" s="5" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>PARTCODR</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>ROPENS</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>1001</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-05</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>EXTRACTED</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>NEW_FILE</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>PARTCODR</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>ROPENS</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>1002</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>2026-01-05</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr">
-        <is>
-          <t>EXTRACTED</t>
-        </is>
-      </c>
-      <c r="H8" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="I8" s="4" t="inlineStr">
-        <is>
-          <t>NEW_FILE</t>
-        </is>
-      </c>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1541,57 +1690,152 @@
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
+          <t>1002</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>EXTRACTED</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O9" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>PARTCODR</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>ROPENS</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
           <t>1003</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>EXTRACTED</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="L10" s="4" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="M10" s="4" t="inlineStr">
         <is>
           <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M9"/>
+  <autoFilter ref="A1:P10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1602,86 +1846,128 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:T5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="46" customWidth="1" min="12" max="12"/>
-    <col width="46" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="46" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
+          <t>Ovrd_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
           <t>Req_ID</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Project_Cd</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Table_Nm</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Src_Cd</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Run_Ty</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Rpt_Start_Dt_Key</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Rpt_End_Dt_Key</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>Btch_ID</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>Used_Btch_ID</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>Override_Ty</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>Prior_Btch_ID</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>Prior_Resolution_Ty</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Apprvl_Stat</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Apprvd_By</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Apprvd_Dtts</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Revoked_By</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>Revoked_Dtts</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>Revocation_Rsn</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>History</t>
         </is>
@@ -1691,163 +1977,328 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_DAILY_2026_1</t>
-        </is>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_DAILY_2026_1</t>
+          <t>PROGAUDIT</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>ODAG1</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
           <t>CARRY_FORWARD_REUSE</t>
         </is>
       </c>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>REVOKED</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>jsmith</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>2026-01-02 09:00:00</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>mgarcia</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-05 07:30:00</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Data quality concern raised before Day 5 run</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Day 1: row created, PENDING_REVIEW | Day 2: UPDATE -&gt; APPROVED by jsmith | Day 5: UPDATE -&gt; REVOKED by mgarcia</t>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: row created, PENDING_REVIEW | Day 2: UPDATE -&gt; APPROVED by jsmith | Day 5: UPDATE -&gt; SUPERSEDED (Anchor from Day 4 batch approved for the same reporting period)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>PROGAUDIT</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>CORRECTION_REOPEN</t>
+          <t>ODAG1</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>2001</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>NEW_FILE</t>
+          <t>CMS</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>CARRY_FORWARD_REUSE</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
           <t>APPROVED</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>jsmith</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-08 10:15:00</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Day 8: row created, PENDING_REVIEW (corrected file received for closed batch) | Day 8: UPDATE -&gt; APPROVED by jsmith</t>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05 09:15:00</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="n"/>
+      <c r="R3" s="2" t="n"/>
+      <c r="S3" s="2" t="n"/>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>Day 4: row created, PENDING_REVIEW | Day 5: UPDATE -&gt; APPROVED by jsmith (previous anchor from Day 1 auto-superseded in the same transaction)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>PARTCODR</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>ROPENS</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>1003</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>CORRECTION_REOPEN</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>jsmith</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-08 10:15:00</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="n"/>
+      <c r="R4" s="2" t="n"/>
+      <c r="S4" s="2" t="n"/>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>Day 8: row created, PENDING_REVIEW (corrected file received for closed batch) | Day 8: UPDATE -&gt; APPROVED by jsmith</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>PARTCODR</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ROPENS</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>1002</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
         <is>
           <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>LATE_ARRIVAL_REOPEN</t>
         </is>
       </c>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="L5" s="2" t="n"/>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>APPROVED</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>jsmith</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="P5" s="2" t="inlineStr">
         <is>
           <t>2026-01-09 11:40:00</t>
         </is>
       </c>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="Q5" s="2" t="n"/>
+      <c r="R5" s="2" t="n"/>
+      <c r="S5" s="2" t="n"/>
+      <c r="T5" s="2" t="inlineStr">
         <is>
           <t>Day 9: row created, PENDING_REVIEW (late file received for closed/missing batch) | Day 9: UPDATE -&gt; APPROVED by jsmith</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M4"/>
+  <autoFilter ref="A1:T5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2083,7 +2534,7 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
@@ -2138,7 +2589,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>20260102_PROGAUDIT_ODAG1_2001_DAILY_2026_1</t>
+          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2168,7 +2619,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>FDR 2001 file not received for Jan 2</t>
+          <t>FDR 2001 no approved anchor available for Jan 2 (Anchor #1 still PENDING_REVIEW at run time)</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2629,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>20260105_PROGAUDIT_ODAG1_2001_DAILY_2026_1</t>
+          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2188,7 +2639,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>CARRY_FORWARD_REVOKED</t>
+          <t>CARRY_FORWARD_ANCHOR_SUPERSEDED</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -2198,17 +2649,17 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>mgarcia</t>
+          <t>jsmith</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-01-05 07:30:00</t>
+          <t>2026-01-05 09:15:00</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Approval revoked for Jan 1 anchor before Day 5 run</t>
+          <t>Anchor #2 (Day 4 batch) approved; Anchor #1 (Day 1 batch) auto-superseded for the same CMS reporting period</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reverse resolution priority (approved anchor wins over new file), add Reuse_Valid_Thru_Dt_Key expiry, gate new anchor creation on revoke, update-in-place for pending candidates
</commit_message>
<xml_diff>
--- a/mock-data/cms_compliance_framework_tables.xlsx
+++ b/mock-data/cms_compliance_framework_tables.xlsx
@@ -21,9 +21,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ComplianceRunType'!$A$1:$C$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ComplianceDataSetSourceXwalk'!$A$1:$F$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ComplianceRequestControl'!$A$1:$P$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ComplianceBatchOverride'!$A$1:$T$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ComplianceBatchOverride'!$A$1:$U$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ComplianceExtractControl'!$A$1:$M$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'CMS_ComplianceExceptionsAudit'!$A$1:$H$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'CMS_ComplianceExceptionsAudit'!$A$1:$H$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -51,7 +51,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -78,14 +78,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
-        <bgColor rgb="00E2EFDA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DDEBF7"/>
-        <bgColor rgb="00DDEBF7"/>
+        <fgColor rgb="00FFF2CC"/>
+        <bgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -115,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -127,7 +121,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -586,7 +579,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Sparse gate for reuse + reopen - one APPROVED row max per project/table/source/run type/reporting period</t>
+          <t>Sparse gate - at most one active (PENDING_REVIEW/APPROVED) row per grouping; Reuse_Valid_Thru_Dt_Key caps how long an approved anchor may be reused</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -616,11 +609,11 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Append-only log - includes upstream-rejected files that never touched CRC/Override</t>
+          <t>Append-only log - includes files received-but-not-promoted and upstream-rejected files</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1199,396 +1192,392 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>PROGAUDIT</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>2001</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>CMS</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>2026-01-02</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>2026-01-31</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>RULES_PASSED</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>PROGAUDIT</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>ODAG1</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>20260103_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>DATA_NOT_PROVIDED</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="M3" s="5" t="n"/>
-      <c r="N3" s="5" t="inlineStr">
+      <c r="M4" s="5" t="n"/>
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="O3" s="5" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>PROGAUDIT</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>2001</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>CMS</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-03</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>2026-01-31</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>20260103_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>EXTRACTED</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>CARRIED_FORWARD</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
+          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L4" s="6" t="inlineStr">
-        <is>
-          <t>CARRIED_FORWARD</t>
-        </is>
-      </c>
-      <c r="M4" s="6" t="inlineStr">
-        <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="N4" s="6" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P5" s="6" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>PROGAUDIT</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>ODAG1</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>CMS</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>20260105_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>DATA_NOT_PROVIDED</t>
+        </is>
+      </c>
+      <c r="K6" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="O4" s="6" t="inlineStr">
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>MISSING</t>
+        </is>
+      </c>
+      <c r="M6" s="5" t="n"/>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="O6" s="5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P4" s="6" t="inlineStr">
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>PROGAUDIT</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>2001</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
           <t>CMS</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>2026-01-04</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>2026-01-31</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
         <is>
           <t>RULES_PASSED</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
-        <is>
-          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="N5" s="4" t="inlineStr">
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="O5" s="4" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P5" s="4" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>PROGAUDIT</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>ODAG1</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>CMS</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-05</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>2026-01-31</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>20260105_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>EXTRACTED</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L6" s="6" t="inlineStr">
-        <is>
-          <t>CARRIED_FORWARD</t>
-        </is>
-      </c>
-      <c r="M6" s="6" t="inlineStr">
-        <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="N6" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O6" s="6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P6" s="6" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>PROGAUDIT</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>ODAG1</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>CMS</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>2026-01-06</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="H7" s="7" t="inlineStr">
-        <is>
-          <t>2026-01-31</t>
-        </is>
-      </c>
-      <c r="I7" s="7" t="inlineStr">
-        <is>
-          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="J7" s="7" t="inlineStr">
-        <is>
-          <t>EXTRACTED</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="L7" s="7" t="inlineStr">
-        <is>
-          <t>CARRIED_FORWARD</t>
-        </is>
-      </c>
-      <c r="M7" s="7" t="inlineStr">
-        <is>
-          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="N7" s="7" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="O7" s="7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="P7" s="7" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1846,7 +1835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1862,13 +1851,14 @@
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="44" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
     <col width="11" customWidth="1" min="15" max="15"/>
     <col width="21" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="46" customWidth="1" min="20" max="20"/>
+    <col width="25" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="21" customWidth="1" min="19" max="19"/>
+    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="46" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1954,20 +1944,25 @@
       </c>
       <c r="Q1" s="3" t="inlineStr">
         <is>
+          <t>Reuse_Valid_Thru_Dt_Key</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
           <t>Revoked_By</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>Revoked_Dtts</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>Revocation_Rsn</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>History</t>
         </is>
@@ -1978,7 +1973,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -2012,12 +2007,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -2029,7 +2024,7 @@
       <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>REVOKED</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -2039,15 +2034,32 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>2026-01-02 09:00:00</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="n"/>
-      <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="n"/>
+          <t>2026-01-03 09:00:00</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>mgarcia</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05 07:30:00</t>
+        </is>
+      </c>
       <c r="T2" s="2" t="inlineStr">
         <is>
-          <t>Day 1: row created, PENDING_REVIEW | Day 2: UPDATE -&gt; APPROVED by jsmith | Day 5: UPDATE -&gt; SUPERSEDED (Anchor from Day 4 batch approved for the same reporting period)</t>
+          <t>Data quality issue found in Day 2 file</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>Day 1: row created, PENDING_REVIEW (candidate: Day 1 batch) | Day 2: candidate replaced with Day 2's batch, still PENDING_REVIEW | Day 3: UPDATE -&gt; APPROVED by jsmith, valid through 2026-01-31 | Day 5: UPDATE -&gt; REVOKED by mgarcia - data quality issue found</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2068,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -2090,12 +2102,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -2107,25 +2119,18 @@
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>APPROVED</t>
-        </is>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>jsmith</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-05 09:15:00</t>
-        </is>
-      </c>
+          <t>PENDING_REVIEW</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="n"/>
       <c r="R3" s="2" t="n"/>
       <c r="S3" s="2" t="n"/>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>Day 4: row created, PENDING_REVIEW | Day 5: UPDATE -&gt; APPROVED by jsmith (previous anchor from Day 1 auto-superseded in the same transaction)</t>
+      <c r="T3" s="2" t="n"/>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>Day 6: row created, PENDING_REVIEW (candidate: Day 6 batch) - grouping was free again after prior anchor's REVOKED status on Day 5</t>
         </is>
       </c>
     </row>
@@ -2209,7 +2214,8 @@
       <c r="Q4" s="2" t="n"/>
       <c r="R4" s="2" t="n"/>
       <c r="S4" s="2" t="n"/>
-      <c r="T4" s="2" t="inlineStr">
+      <c r="T4" s="2" t="n"/>
+      <c r="U4" s="2" t="inlineStr">
         <is>
           <t>Day 8: row created, PENDING_REVIEW (corrected file received for closed batch) | Day 8: UPDATE -&gt; APPROVED by jsmith</t>
         </is>
@@ -2291,14 +2297,15 @@
       <c r="Q5" s="2" t="n"/>
       <c r="R5" s="2" t="n"/>
       <c r="S5" s="2" t="n"/>
-      <c r="T5" s="2" t="inlineStr">
+      <c r="T5" s="2" t="n"/>
+      <c r="U5" s="2" t="inlineStr">
         <is>
           <t>Day 9: row created, PENDING_REVIEW (late file received for closed/missing batch) | Day 9: UPDATE -&gt; APPROVED by jsmith</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T5"/>
+  <autoFilter ref="A1:U5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2528,13 +2535,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
@@ -2589,7 +2596,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+          <t>20260103_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2614,12 +2621,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>2026-01-02 20:00:00</t>
+          <t>2026-01-03 20:00:00</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>FDR 2001 no approved anchor available for Jan 2 (Anchor #1 still PENDING_REVIEW at run time)</t>
+          <t>FDR 2001 no approved anchor available for Jan 3 (candidate still PENDING_REVIEW at run time)</t>
         </is>
       </c>
     </row>
@@ -2639,7 +2646,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>CARRY_FORWARD_ANCHOR_SUPERSEDED</t>
+          <t>FILE_RECEIVED_ANCHOR_ACTIVE</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -2649,17 +2656,17 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>jsmith</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-01-05 09:15:00</t>
+          <t>2026-01-04 06:00:00</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Anchor #2 (Day 4 batch) approved; Anchor #1 (Day 1 batch) auto-superseded for the same CMS reporting period</t>
+          <t>File received for Jan 4 but NOT promoted - approved anchor (Day 2 batch) still active and valid through 2026-01-31; anchor must be revoked before a new file can be considered</t>
         </is>
       </c>
     </row>
@@ -2667,35 +2674,39 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="n"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>EXCEPTION</t>
+          <t>AUDIT</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>DUPLICATE_FILE_IGNORED</t>
+          <t>CARRY_FORWARD_ANCHOR_REVOKED</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>WARNING</t>
+          <t>INFO</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>SYSTEM</t>
+          <t>mgarcia</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>2026-01-07 08:00:00</t>
+          <t>2026-01-05 07:30:00</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Duplicate resend of 1001's Jan 5 file - checksum matched, quarantined, no CRC/Override write</t>
+          <t>Anchor (Day 2 batch) revoked - data quality issue found; grouping now open for a new anchor</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2722,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>UNRECOGNIZED_SOURCE</t>
+          <t>DUPLICATE_FILE_IGNORED</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -2726,12 +2737,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-01-07 08:05:00</t>
+          <t>2026-01-07 08:00:00</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>File from src=9999 not in ComplianceDataSetSourceXwalk - quarantined, no CRC/Override write</t>
+          <t>Duplicate resend of 1001's Jan 5 file - checksum matched, quarantined, no CRC/Override write</t>
         </is>
       </c>
     </row>
@@ -2739,39 +2750,35 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
+      <c r="B6" s="2" t="n"/>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>AUDIT</t>
+          <t>EXCEPTION</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>CORRECTION_REOPEN_APPROVED</t>
+          <t>UNRECOGNIZED_SOURCE</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>jsmith</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-01-08 10:15:00</t>
+          <t>2026-01-07 08:05:00</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Corrected file accepted for 1003, Jan 5 - CRC row and extract reopened/reclosed</t>
+          <t>File from src=9999 not in ComplianceDataSetSourceXwalk - quarantined, no CRC/Override write</t>
         </is>
       </c>
     </row>
@@ -2781,42 +2788,82 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
+          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>CORRECTION_REOPEN_APPROVED</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>jsmith</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-08 10:15:00</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Corrected file accepted for 1003, Jan 5 - CRC row and extract reopened/reclosed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
           <t>20260106_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>AUDIT</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>LATE_ARRIVAL_REOPEN_APPROVED</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>INFO</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>jsmith</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>2026-01-09 11:40:00</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Late file accepted for 1002, Jan 5 (4 days late) - CRC row and extract reopened/reclosed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H7"/>
+  <autoFilter ref="A1:H8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Consolidate into framework-master.md: full requirements, final DDLs, end-to-end pipeline, and a failure-points review (3 gaps found and closed)
</commit_message>
<xml_diff>
--- a/mock-data/cms_compliance_framework_tables.xlsx
+++ b/mock-data/cms_compliance_framework_tables.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ComplianceSourceSystem'!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ComplianceRunType'!$A$1:$C$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ComplianceDataSetSourceXwalk'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ComplianceRequestControl'!$A$1:$P$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ComplianceRequestControl'!$A$1:$Q$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ComplianceBatchOverride'!$A$1:$U$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ComplianceExtractControl'!$A$1:$M$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'CMS_ComplianceExceptionsAudit'!$A$1:$H$8</definedName>
@@ -564,7 +564,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CRC - one row per source/table/run type/date, current-state, updated in place</t>
+          <t>CRC - one row per source/table/run type/date, current-state; Received_File_Ref logs every arrival, promoted or not (G1 fix)</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -579,7 +579,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Sparse gate - at most one active (PENDING_REVIEW/APPROVED) row per grouping; Reuse_Valid_Thru_Dt_Key caps how long an approved anchor may be reused</t>
+          <t>Sparse gate - at most one active row per grouping; Reuse_Valid_Thru_Dt_Key required on approval (G3 fix)</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -609,7 +609,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Append-only log - includes files received-but-not-promoted and upstream-rejected files</t>
+          <t>Append-only log - files received-but-not-promoted, upstream-rejected files, and all approval/revoke/expiry events</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -1008,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1022,11 +1022,12 @@
     <col width="44" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="44" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="46" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1087,25 +1088,30 @@
       </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
+          <t>Received_File_Ref</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
           <t>Resolution_Ty</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>Used_Btch_ID</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Late_Arrival_Ind</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Batch_Close_Ind</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Batch_Closed_By</t>
         </is>
@@ -1167,25 +1173,30 @@
       </c>
       <c r="L2" s="4" t="inlineStr">
         <is>
+          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260101.dat</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1247,25 +1258,30 @@
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
+          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260102.dat</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="Q3" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1325,23 +1341,24 @@
           <t>N</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L4" s="5" t="n"/>
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="M4" s="5" t="n"/>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N4" s="5" t="n"/>
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="Q4" s="5" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1403,25 +1420,30 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
+          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260104.dat  (received, NOT promoted - see G1)</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
           <t>CARRIED_FORWARD</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
-      <c r="N5" s="6" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="O5" s="6" t="inlineStr">
+      <c r="P5" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P5" s="6" t="inlineStr">
+      <c r="Q5" s="6" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1481,23 +1503,24 @@
           <t>N</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr">
+      <c r="L6" s="5" t="n"/>
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="M6" s="5" t="n"/>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="N6" s="5" t="n"/>
+      <c r="O6" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr">
+      <c r="Q6" s="5" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1559,25 +1582,30 @@
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
+          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260106.dat</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P7" s="4" t="inlineStr">
+      <c r="Q7" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1639,25 +1667,30 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1001/20260106.dat</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="Q8" s="2" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1719,25 +1752,30 @@
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1002/20260109.dat</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
+      <c r="P9" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P9" s="4" t="inlineStr">
+      <c r="Q9" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1799,32 +1837,37 @@
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1003/20260108.dat</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="P10" s="4" t="inlineStr">
+      <c r="Q10" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P10"/>
+  <autoFilter ref="A1:Q10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2130,7 +2173,7 @@
       <c r="T3" s="2" t="n"/>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>Day 6: row created, PENDING_REVIEW (candidate: Day 6 batch) - grouping was free again after prior anchor's REVOKED status on Day 5</t>
+          <t>Day 6: row created, PENDING_REVIEW (candidate: Day 6 batch) - grouping free again after Day 5 revoke. Note: Day 4's received-but-ignored file (see CRC Received_File_Ref) remained available as a recovery candidate too, per the G1 fix, had no fresh file arrived by Day 6</t>
         </is>
       </c>
     </row>
@@ -2666,7 +2709,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>File received for Jan 4 but NOT promoted - approved anchor (Day 2 batch) still active and valid through 2026-01-31; anchor must be revoked before a new file can be considered</t>
+          <t>File received for Jan 4 (see Received_File_Ref) but NOT promoted - approved anchor (Day 2 batch) still active and valid through 2026-01-31; stored for recovery per G1 if the anchor is later revoked</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clarify G1 (loaded-but-not-promoted, never feeds extract), add orchestration-flow.md with diagrams + AWS service mapping
</commit_message>
<xml_diff>
--- a/mock-data/cms_compliance_framework_tables.xlsx
+++ b/mock-data/cms_compliance_framework_tables.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ComplianceSourceSystem'!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ComplianceRunType'!$A$1:$C$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ComplianceDataSetSourceXwalk'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ComplianceRequestControl'!$A$1:$Q$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ComplianceRequestControl'!$A$1:$R$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ComplianceBatchOverride'!$A$1:$U$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ComplianceExtractControl'!$A$1:$M$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'CMS_ComplianceExceptionsAudit'!$A$1:$H$8</definedName>
@@ -564,7 +564,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CRC - one row per source/table/run type/date, current-state; Received_File_Ref logs every arrival, promoted or not (G1 fix)</t>
+          <t>CRC - one row per source/table/run type/date, current-state; Received_File_Ref + Received_File_Loaded_Ind log every arrival, even one loaded to staging but never promoted to Used_Btch_ID (G1 fix)</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -1008,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1023,7 +1023,7 @@
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="19" customWidth="1" min="11" max="11"/>
     <col width="46" customWidth="1" min="12" max="12"/>
-    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
     <col width="44" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
@@ -1093,25 +1093,30 @@
       </c>
       <c r="M1" s="3" t="inlineStr">
         <is>
+          <t>Received_File_Loaded_Ind</t>
+        </is>
+      </c>
+      <c r="N1" s="3" t="inlineStr">
+        <is>
           <t>Resolution_Ty</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>Used_Btch_ID</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Late_Arrival_Ind</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>Batch_Close_Ind</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>Batch_Closed_By</t>
         </is>
@@ -1176,27 +1181,32 @@
           <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260101.dat</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
-      <c r="O2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="Q2" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1261,27 +1271,32 @@
           <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260102.dat</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
-      <c r="O3" s="4" t="inlineStr">
+      <c r="P3" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1342,23 +1357,28 @@
         </is>
       </c>
       <c r="L4" s="5" t="n"/>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="N4" s="5" t="n"/>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O4" s="5" t="n"/>
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R4" s="5" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1423,27 +1443,32 @@
           <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260104.dat  (received, NOT promoted - see G1)</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>CARRIED_FORWARD</t>
         </is>
       </c>
-      <c r="N5" s="6" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
-      <c r="O5" s="6" t="inlineStr">
+      <c r="P5" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="P5" s="6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="Q5" s="6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R5" s="6" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1504,23 +1529,28 @@
         </is>
       </c>
       <c r="L6" s="5" t="n"/>
-      <c r="M6" s="5" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="N6" s="5" t="n"/>
-      <c r="O6" s="5" t="inlineStr">
+      <c r="O6" s="5" t="n"/>
+      <c r="P6" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="P6" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="Q6" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1585,27 +1615,32 @@
           <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260106.dat</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N7" s="4" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="O7" s="4" t="inlineStr">
         <is>
           <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
         </is>
       </c>
-      <c r="O7" s="4" t="inlineStr">
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="P7" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R7" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1672,25 +1707,30 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="N8" s="2" t="inlineStr">
+      <c r="O8" s="2" t="inlineStr">
         <is>
           <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
         </is>
       </c>
-      <c r="O8" s="2" t="inlineStr">
+      <c r="P8" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1755,27 +1795,32 @@
           <t>s3://cms-inbound/PARTCODR/ROPENS/1002/20260109.dat</t>
         </is>
       </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N9" s="4" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="O9" s="4" t="inlineStr">
         <is>
           <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
         </is>
       </c>
-      <c r="O9" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
       <c r="Q9" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R9" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1840,34 +1885,39 @@
           <t>s3://cms-inbound/PARTCODR/ROPENS/1003/20260108.dat</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="P10" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
       <c r="Q10" s="4" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R10" s="4" t="inlineStr">
+        <is>
           <t>SYSTEM</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q10"/>
+  <autoFilter ref="A1:R10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Rebuild Part C ODR mock data: 3 FDRs required per date across 2 dates - missing/late-arrival case (Jan 5) and incorrect/correction case (Jan 12)
</commit_message>
<xml_diff>
--- a/mock-data/cms_compliance_framework_tables.xlsx
+++ b/mock-data/cms_compliance_framework_tables.xlsx
@@ -20,10 +20,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ComplianceSourceSystem'!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ComplianceRunType'!$A$1:$C$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ComplianceDataSetSourceXwalk'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ComplianceRequestControl'!$A$1:$R$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ComplianceRequestControl'!$A$1:$R$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ComplianceBatchOverride'!$A$1:$U$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ComplianceExtractControl'!$A$1:$M$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'CMS_ComplianceExceptionsAudit'!$A$1:$H$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ComplianceExtractControl'!$A$1:$M$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'CMS_ComplianceExceptionsAudit'!$A$1:$H$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -564,11 +564,11 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CRC - one row per source/table/run type/date, current-state; Received_File_Ref + Received_File_Loaded_Ind log every arrival, even one loaded to staging but never promoted to Used_Btch_ID (G1 fix)</t>
+          <t>CRC - one row per source/table/run type/date, current-state; Part C ODR section now covers 2 dates x 3 required FDRs each</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -579,7 +579,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Sparse gate - at most one active row per grouping; Reuse_Valid_Thru_Dt_Key required on approval (G3 fix)</t>
+          <t>Sparse gate - carry-forward reuse (Example A) + late-arrival and correction reopen (Example B, 2 dates)</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -594,11 +594,11 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>One row per table/date - tracks PARTIAL/COMPLETE and the close/reopen lock</t>
+          <t>One row per table/date - PARTIAL-&gt;COMPLETE (missing-FDR case) and COMPLETE-&gt;COMPLETE-with-corrected-batch (incorrect-data case)</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -609,11 +609,11 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Append-only log - files received-but-not-promoted, upstream-rejected files, and all approval/revoke/expiry events</t>
+          <t>Append-only log - missing/incorrect-data flags, reopen approvals, upstream-rejected files</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1008,7 +1008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1024,10 +1024,11 @@
     <col width="19" customWidth="1" min="11" max="11"/>
     <col width="46" customWidth="1" min="12" max="12"/>
     <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="44" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="44" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
     <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1181,9 +1182,9 @@
           <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260101.dat</t>
         </is>
       </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
       <c r="N2" s="4" t="inlineStr">
@@ -1271,9 +1272,9 @@
           <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260102.dat</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
@@ -1357,7 +1358,7 @@
         </is>
       </c>
       <c r="L4" s="5" t="n"/>
-      <c r="M4" s="2" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1440,10 +1441,10 @@
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260104.dat  (received, NOT promoted - see G1)</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
+          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260104.dat</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1529,7 +1530,7 @@
         </is>
       </c>
       <c r="L6" s="5" t="n"/>
-      <c r="M6" s="2" t="inlineStr">
+      <c r="M6" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -1615,9 +1616,9 @@
           <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260106.dat</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
@@ -1707,7 +1708,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1795,7 +1796,7 @@
           <t>s3://cms-inbound/PARTCODR/ROPENS/1002/20260109.dat</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr">
+      <c r="M9" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1827,97 +1828,367 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n">
+      <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>PARTCODR</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>ROPENS</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>1003</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>DAILY</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
         <is>
           <t>EXTRACTED</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PARTCODR/ROPENS/1003/20260108.dat</t>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1003/20260106.dat</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N10" s="4" t="inlineStr">
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="O10" s="4" t="inlineStr">
-        <is>
-          <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="P10" s="4" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="Q10" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="R10" s="4" t="inlineStr">
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>PARTCODR</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>ROPENS</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>1001</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>20260113_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACTED</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1001/20260113.dat</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>20260113_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>PARTCODR</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>ROPENS</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>1002</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>20260113_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>EXTRACTED</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1002/20260113.dat</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>20260113_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>PARTCODR</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>ROPENS</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>1003</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>DAILY</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>EXTRACTED</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1003/20260116.dat</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="O13" s="4" t="inlineStr">
+        <is>
+          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="R13" s="4" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R10"/>
+  <autoFilter ref="A1:R13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2223,7 +2494,7 @@
       <c r="T3" s="2" t="n"/>
       <c r="U3" s="2" t="inlineStr">
         <is>
-          <t>Day 6: row created, PENDING_REVIEW (candidate: Day 6 batch) - grouping free again after Day 5 revoke. Note: Day 4's received-but-ignored file (see CRC Received_File_Ref) remained available as a recovery candidate too, per the G1 fix, had no fresh file arrived by Day 6</t>
+          <t>Day 6: row created, PENDING_REVIEW (candidate: Day 6 batch) - grouping free again after Day 5 revoke. Note: Day 4's received-but-loaded file remained available as a recovery candidate too, per the G1 fix, had no fresh file arrived by Day 6</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2503,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -2246,7 +2517,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>1002</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -2266,27 +2537,23 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>CORRECTION_REOPEN</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
+          <t>LATE_ARRIVAL_REOPEN</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="n"/>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>NEW_FILE</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -2301,7 +2568,7 @@
       </c>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>2026-01-08 10:15:00</t>
+          <t>2026-01-09 11:40:00</t>
         </is>
       </c>
       <c r="Q4" s="2" t="n"/>
@@ -2310,7 +2577,7 @@
       <c r="T4" s="2" t="n"/>
       <c r="U4" s="2" t="inlineStr">
         <is>
-          <t>Day 8: row created, PENDING_REVIEW (corrected file received for closed batch) | Day 8: UPDATE -&gt; APPROVED by jsmith</t>
+          <t>Jan 9: row created, PENDING_REVIEW (late file received for closed/missing batch, Jan 5, 3 days late) | Jan 9: UPDATE -&gt; APPROVED by jsmith</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2586,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -2333,7 +2600,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>1003</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -2343,33 +2610,37 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>2026-01-05</t>
+          <t>2026-01-12</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>LATE_ARRIVAL_REOPEN</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="n"/>
+          <t>CORRECTION_REOPEN</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>20260113_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>MISSING</t>
+          <t>NEW_FILE</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -2384,7 +2655,7 @@
       </c>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>2026-01-09 11:40:00</t>
+          <t>2026-01-16 10:15:00</t>
         </is>
       </c>
       <c r="Q5" s="2" t="n"/>
@@ -2393,7 +2664,7 @@
       <c r="T5" s="2" t="n"/>
       <c r="U5" s="2" t="inlineStr">
         <is>
-          <t>Day 9: row created, PENDING_REVIEW (late file received for closed/missing batch) | Day 9: UPDATE -&gt; APPROVED by jsmith</t>
+          <t>Jan 16: row created, PENDING_REVIEW (corrected file received for closed batch, Jan 12 - original file's data was found incorrect on Jan 14 review) | Jan 16: UPDATE -&gt; APPROVED by jsmith</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2612,12 +2883,77 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Reopened twice: 1003 correction approved Jan 8, then 1002 late arrival approved Jan 9</t>
+          <t>1002 missing at Jan 6 close (PARTIAL, [1001,1003]) - late arrival approved Jan 9, regenerated COMPLETE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>PARTCODR</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>ROPENS</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>COMPLETE</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>[1001,1002,1003]</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16 11:00:00</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>jsmith</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>All 3 FDRs present at Jan 13 close (COMPLETE) but 1003's data was later found incorrect - correction approved Jan 16, regenerated with the corrected 1003 batch. Close/reopen applies regardless of whether the extract was PARTIAL or COMPLETE when it closed.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M3"/>
+  <autoFilter ref="A1:M4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2628,7 +2964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2759,7 +3095,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>File received for Jan 4 (see Received_File_Ref) but NOT promoted - approved anchor (Day 2 batch) still active and valid through 2026-01-31; stored for recovery per G1 if the anchor is later revoked</t>
+          <t>File received and loaded for Jan 4 but NOT used for the extract - approved anchor (Day 2 batch) still active and valid through 2026-01-31</t>
         </is>
       </c>
     </row>
@@ -2807,7 +3143,11 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="n"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
           <t>EXCEPTION</t>
@@ -2815,7 +3155,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>DUPLICATE_FILE_IGNORED</t>
+          <t>SOURCE_MISSING_AT_COMBINE</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -2830,12 +3170,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>2026-01-07 08:00:00</t>
+          <t>2026-01-06 20:00:00</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Duplicate resend of 1001's Jan 5 file - checksum matched, quarantined, no CRC/Override write</t>
+          <t>FDR 1002 file not received for Jan 5 by SLA cutoff - extract closed PARTIAL, [1001,1003] only</t>
         </is>
       </c>
     </row>
@@ -2851,7 +3191,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>UNRECOGNIZED_SOURCE</t>
+          <t>DUPLICATE_FILE_IGNORED</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -2866,12 +3206,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>2026-01-07 08:05:00</t>
+          <t>2026-01-07 08:00:00</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>File from src=9999 not in ComplianceDataSetSourceXwalk - quarantined, no CRC/Override write</t>
+          <t>Duplicate resend of 1001's Jan 5 file - checksum matched, quarantined, no CRC/Override write</t>
         </is>
       </c>
     </row>
@@ -2879,39 +3219,35 @@
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
+      <c r="B7" s="2" t="n"/>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>AUDIT</t>
+          <t>EXCEPTION</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>CORRECTION_REOPEN_APPROVED</t>
+          <t>UNRECOGNIZED_SOURCE</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>INFO</t>
+          <t>WARNING</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>jsmith</t>
+          <t>SYSTEM</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>2026-01-08 10:15:00</t>
+          <t>2026-01-07 08:05:00</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Corrected file accepted for 1003, Jan 5 - CRC row and extract reopened/reclosed</t>
+          <t>File from src=9999 not in ComplianceDataSetSourceXwalk - quarantined, no CRC/Override write</t>
         </is>
       </c>
     </row>
@@ -2921,7 +3257,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>20260106_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2951,12 +3287,92 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Late file accepted for 1002, Jan 5 (4 days late) - CRC row and extract reopened/reclosed</t>
+          <t>Late file accepted for 1002, Jan 5 (3 days late) - CRC row and extract reopened/regenerated/reclosed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>20260113_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>EXCEPTION</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>DATA_QUALITY_ISSUE_FLAGGED</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>mgarcia</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14 13:00:00</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>1003's Jan 12 file passed rules validation but was found to contain incorrect data on manual review - corrected file requested from vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>CORRECTION_REOPEN_APPROVED</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>jsmith</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16 10:15:00</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Corrected file accepted for 1003, Jan 12 - CRC row and extract reopened/regenerated/reclosed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H8"/>
+  <autoFilter ref="A1:H10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add G4: manual data-quality flag path via ComplianceRequestInTake + CRC Flagged_For_Correction_Ind, separate from the automatic reopen mechanism
</commit_message>
<xml_diff>
--- a/mock-data/cms_compliance_framework_tables.xlsx
+++ b/mock-data/cms_compliance_framework_tables.xlsx
@@ -11,19 +11,21 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceSourceSystem" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceRunType" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceDataSetSourceXwalk" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceRequestControl" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceBatchOverride" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceExtractControl" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CMS_ComplianceExceptionsAudit" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceRequestInTake" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceRequestControl" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceBatchOverride" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceExtractControl" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CMS_ComplianceExceptionsAudit" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ComplianceSourceSystem'!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ComplianceRunType'!$A$1:$C$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ComplianceDataSetSourceXwalk'!$A$1:$F$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ComplianceRequestControl'!$A$1:$R$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ComplianceBatchOverride'!$A$1:$U$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ComplianceExtractControl'!$A$1:$M$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'CMS_ComplianceExceptionsAudit'!$A$1:$H$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ComplianceRequestInTake'!$A$1:$K$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ComplianceRequestControl'!$A$1:$V$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ComplianceBatchOverride'!$A$1:$U$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'ComplianceExtractControl'!$A$1:$M$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'CMS_ComplianceExceptionsAudit'!$A$1:$H$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -486,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -559,60 +561,75 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ComplianceRequestControl</t>
+          <t>ComplianceRequestInTake</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>CRC - one row per source/table/run type/date, current-state; Part C ODR section now covers 2 dates x 3 required FDRs each</t>
+          <t>The one table a human writes to directly - data-quality flags (G4) and other genuinely business-initiated asks</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ComplianceBatchOverride</t>
+          <t>ComplianceRequestControl</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Sparse gate - carry-forward reuse (Example A) + late-arrival and correction reopen (Example B, 2 dates)</t>
+          <t>CRC - one row per source/table/run type/date, current-state; Flagged_For_Correction_Ind shows a business flag is open, separate from Override</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ComplianceExtractControl</t>
+          <t>ComplianceBatchOverride</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>One row per table/date - PARTIAL-&gt;COMPLETE (missing-FDR case) and COMPLETE-&gt;COMPLETE-with-corrected-batch (incorrect-data case)</t>
+          <t>Sparse gate - carry-forward reuse (Example A) + late-arrival and correction reopen (Example B, 2 dates)</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>ComplianceExtractControl</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>One row per table/date - PARTIAL-&gt;COMPLETE and COMPLETE-&gt;COMPLETE-with-corrected-batch reopen cases</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>CMS_ComplianceExceptionsAudit</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Append-only log - missing/incorrect-data flags, reopen approvals, upstream-rejected files</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Append-only log - data-quality flags, reopen approvals, upstream-rejected files</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
         <v>9</v>
       </c>
     </row>
@@ -1008,7 +1025,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Intake_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Project_Cd</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Table_Nm</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Src_Cd</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Req_Dt_Key</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Req_Ty</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Requested_By</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Requested_Dtts</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Rsn</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Processed_Ind</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>Processed_Dtts</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>INT-0001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>PARTCODR</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>ROPENS</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>1003</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>CORRECTION_REQUEST</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>mgarcia</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14 13:00:00</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>1003's Jan 12 file passed rules validation but manual review found incorrect data - requesting corrected file from vendor</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14 13:05:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1027,8 +1186,10 @@
     <col width="17" customWidth="1" min="14" max="14"/>
     <col width="44" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="17" customWidth="1" min="17" max="17"/>
-    <col width="17" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="22" customWidth="1" min="18" max="18"/>
+    <col width="22" customWidth="1" min="19" max="19"/>
+    <col width="22" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1114,10 +1275,30 @@
       </c>
       <c r="Q1" s="3" t="inlineStr">
         <is>
+          <t>Flagged_For_Correction_Ind</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>Flagged_By</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>Flagged_Dtts</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>Flag_Rsn</t>
+        </is>
+      </c>
+      <c r="U1" s="3" t="inlineStr">
+        <is>
           <t>Batch_Close_Ind</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>Batch_Closed_By</t>
         </is>
@@ -1202,12 +1383,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="R2" s="4" t="inlineStr">
+      <c r="V2" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1292,12 +1481,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="n"/>
+      <c r="S3" s="2" t="n"/>
+      <c r="T3" s="2" t="n"/>
+      <c r="U3" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="R3" s="4" t="inlineStr">
+      <c r="V3" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1374,12 +1571,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="n"/>
+      <c r="S4" s="2" t="n"/>
+      <c r="T4" s="2" t="n"/>
+      <c r="U4" s="5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="V4" s="5" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1464,12 +1669,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q5" s="6" t="inlineStr">
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="n"/>
+      <c r="S5" s="2" t="n"/>
+      <c r="T5" s="2" t="n"/>
+      <c r="U5" s="6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="R5" s="6" t="inlineStr">
+      <c r="V5" s="6" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1546,12 +1759,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q6" s="5" t="inlineStr">
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="n"/>
+      <c r="S6" s="2" t="n"/>
+      <c r="T6" s="2" t="n"/>
+      <c r="U6" s="5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="R6" s="5" t="inlineStr">
+      <c r="V6" s="5" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1636,12 +1857,20 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q7" s="4" t="inlineStr">
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="n"/>
+      <c r="S7" s="2" t="n"/>
+      <c r="T7" s="2" t="n"/>
+      <c r="U7" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="R7" s="4" t="inlineStr">
+      <c r="V7" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1728,10 +1957,18 @@
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="n"/>
+      <c r="S8" s="2" t="n"/>
+      <c r="T8" s="2" t="n"/>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="R8" s="2" t="inlineStr">
+      <c r="V8" s="2" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1816,12 +2053,20 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="Q9" s="4" t="inlineStr">
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="n"/>
+      <c r="S9" s="2" t="n"/>
+      <c r="T9" s="2" t="n"/>
+      <c r="U9" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="R9" s="4" t="inlineStr">
+      <c r="V9" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1908,10 +2153,18 @@
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="n"/>
+      <c r="S10" s="2" t="n"/>
+      <c r="T10" s="2" t="n"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="R10" s="2" t="inlineStr">
+      <c r="V10" s="2" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -1998,10 +2251,18 @@
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="n"/>
+      <c r="S11" s="2" t="n"/>
+      <c r="T11" s="2" t="n"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="R11" s="2" t="inlineStr">
+      <c r="V11" s="2" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -2088,10 +2349,18 @@
       </c>
       <c r="Q12" s="2" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="n"/>
+      <c r="S12" s="2" t="n"/>
+      <c r="T12" s="2" t="n"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="R12" s="2" t="inlineStr">
+      <c r="V12" s="2" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
@@ -2176,24 +2445,44 @@
           <t>N</t>
         </is>
       </c>
-      <c r="Q13" s="4" t="inlineStr">
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>mgarcia</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14 13:00:00 (cleared 2026-01-16)</t>
+        </is>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>Corrected file approved Jan 16 - flag resolved</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="R13" s="4" t="inlineStr">
+      <c r="V13" s="4" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R13"/>
+  <autoFilter ref="A1:V13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2674,7 +2963,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2958,7 +3247,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
G5: slim CRC to decision-relevant columns only; move file-event detail (received/loaded/late/closed/flagged) into new append-only ComplianceRequestFileDetail, joined on Req_ID
</commit_message>
<xml_diff>
--- a/mock-data/cms_compliance_framework_tables.xlsx
+++ b/mock-data/cms_compliance_framework_tables.xlsx
@@ -13,19 +13,21 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceDataSetSourceXwalk" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceRequestInTake" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceRequestControl" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceBatchOverride" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceExtractControl" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CMS_ComplianceExceptionsAudit" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceRequestFileDetail" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceBatchOverride" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ComplianceExtractControl" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CMS_ComplianceExceptionsAudit" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ComplianceSourceSystem'!$A$1:$D$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'ComplianceRunType'!$A$1:$C$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ComplianceDataSetSourceXwalk'!$A$1:$F$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ComplianceRequestInTake'!$A$1:$K$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ComplianceRequestControl'!$A$1:$V$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ComplianceBatchOverride'!$A$1:$U$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'ComplianceExtractControl'!$A$1:$M$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'CMS_ComplianceExceptionsAudit'!$A$1:$H$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'ComplianceRequestControl'!$A$1:$O$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'ComplianceRequestFileDetail'!$A$1:$J$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'ComplianceBatchOverride'!$A$1:$U$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'ComplianceExtractControl'!$A$1:$M$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'CMS_ComplianceExceptionsAudit'!$A$1:$H$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -488,7 +490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -581,7 +583,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>CRC - one row per source/table/run type/date, current-state; Flagged_For_Correction_Ind shows a business flag is open, separate from Override</t>
+          <t>CRC - kept minimal (G5): only columns the pipeline reads to decide something. One row per source/table/run type/date, current-state</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -591,49 +593,483 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ComplianceBatchOverride</t>
+          <t>ComplianceRequestFileDetail</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Sparse gate - carry-forward reuse (Example A) + late-arrival and correction reopen (Example B, 2 dates)</t>
+          <t>NEW (G5) - append-only file-event log per Req_ID (received, loaded-not-promoted, late arrival, closed, flagged/cleared); join to CRC on Req_ID for detail</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>4</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ComplianceExtractControl</t>
+          <t>ComplianceBatchOverride</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>One row per table/date - PARTIAL-&gt;COMPLETE and COMPLETE-&gt;COMPLETE-with-corrected-batch reopen cases</t>
+          <t>Sparse gate - carry-forward reuse (Example A) + late-arrival and correction reopen (Example B, 2 dates)</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>ComplianceExtractControl</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>One row per table/date - PARTIAL-&gt;COMPLETE and COMPLETE-&gt;COMPLETE-with-corrected-batch reopen cases</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>CMS_ComplianceExceptionsAudit</t>
         </is>
       </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Append-only narrative log - data-quality flags, reopen approvals, upstream-rejected files</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Event_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Btch_ID</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Event_Ctgy</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Event_Ty</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Sevrty</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Event_Dtts</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>20260103_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>EXCEPTION</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>SOURCE_MISSING_AT_COMBINE</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-03 20:00:00</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>FDR 2001 no approved anchor available for Jan 3 (candidate still PENDING_REVIEW at run time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>FILE_RECEIVED_ANCHOR_ACTIVE</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-04 06:00:00</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>File received and loaded for Jan 4 but NOT used for the extract - approved anchor (Day 2 batch) still active and valid through 2026-01-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>CARRY_FORWARD_ANCHOR_REVOKED</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>mgarcia</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-05 07:30:00</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Anchor (Day 2 batch) revoked - data quality issue found; grouping now open for a new anchor</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>EXCEPTION</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>SOURCE_MISSING_AT_COMBINE</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-06 20:00:00</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>FDR 1002 file not received for Jan 5 by SLA cutoff - extract closed PARTIAL, [1001,1003] only</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="n"/>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>EXCEPTION</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>DUPLICATE_FILE_IGNORED</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07 08:00:00</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Duplicate resend of 1001's Jan 5 file - checksum matched, quarantined, no CRC/Override write</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>EXCEPTION</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>UNRECOGNIZED_SOURCE</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-07 08:05:00</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>File from src=9999 not in ComplianceDataSetSourceXwalk - quarantined, no CRC/Override write</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>LATE_ARRIVAL_REOPEN_APPROVED</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>jsmith</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-09 11:40:00</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Late file accepted for 1002, Jan 5 (3 days late) - CRC row and extract reopened/regenerated/reclosed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Append-only log - data-quality flags, reopen approvals, upstream-rejected files</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="n">
+          <t>20260113_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>EXCEPTION</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>DATA_QUALITY_ISSUE_FLAGGED</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>mgarcia</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14 13:00:00</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>1003's Jan 12 file passed rules validation but was found to contain incorrect data on manual review - corrected file requested from vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>AUDIT</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>CORRECTION_REOPEN_APPROVED</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>jsmith</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16 10:15:00</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Corrected file accepted for 1003, Jan 12 - CRC row and extract reopened/regenerated/reclosed</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1167,7 +1603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1180,16 +1616,11 @@
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="44" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
-    <col width="46" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="17" customWidth="1" min="14" max="14"/>
-    <col width="44" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="22" customWidth="1" min="17" max="17"/>
-    <col width="22" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -1245,62 +1676,27 @@
       </c>
       <c r="K1" s="3" t="inlineStr">
         <is>
-          <t>File_Received_Ind</t>
+          <t>Resolution_Ty</t>
         </is>
       </c>
       <c r="L1" s="3" t="inlineStr">
         <is>
-          <t>Received_File_Ref</t>
+          <t>Used_Btch_ID</t>
         </is>
       </c>
       <c r="M1" s="3" t="inlineStr">
         <is>
-          <t>Received_File_Loaded_Ind</t>
+          <t>Batch_Close_Ind</t>
         </is>
       </c>
       <c r="N1" s="3" t="inlineStr">
         <is>
-          <t>Resolution_Ty</t>
+          <t>Created_Dtts</t>
         </is>
       </c>
       <c r="O1" s="3" t="inlineStr">
         <is>
-          <t>Used_Btch_ID</t>
-        </is>
-      </c>
-      <c r="P1" s="3" t="inlineStr">
-        <is>
-          <t>Late_Arrival_Ind</t>
-        </is>
-      </c>
-      <c r="Q1" s="3" t="inlineStr">
-        <is>
-          <t>Flagged_For_Correction_Ind</t>
-        </is>
-      </c>
-      <c r="R1" s="3" t="inlineStr">
-        <is>
-          <t>Flagged_By</t>
-        </is>
-      </c>
-      <c r="S1" s="3" t="inlineStr">
-        <is>
-          <t>Flagged_Dtts</t>
-        </is>
-      </c>
-      <c r="T1" s="3" t="inlineStr">
-        <is>
-          <t>Flag_Rsn</t>
-        </is>
-      </c>
-      <c r="U1" s="3" t="inlineStr">
-        <is>
-          <t>Batch_Close_Ind</t>
-        </is>
-      </c>
-      <c r="V1" s="3" t="inlineStr">
-        <is>
-          <t>Batch_Closed_By</t>
+          <t>Updated_Dtts</t>
         </is>
       </c>
     </row>
@@ -1355,52 +1751,21 @@
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260101.dat</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N2" s="4" t="inlineStr">
-        <is>
-          <t>NEW_FILE</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
-        <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="n"/>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="n"/>
-      <c r="U2" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V2" s="4" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
+      <c r="N2" s="4" t="n"/>
+      <c r="O2" s="4" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -1453,52 +1818,21 @@
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260102.dat</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t>NEW_FILE</t>
-        </is>
-      </c>
-      <c r="O3" s="4" t="inlineStr">
-        <is>
-          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="P3" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="n"/>
-      <c r="S3" s="2" t="n"/>
-      <c r="T3" s="2" t="n"/>
-      <c r="U3" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V3" s="4" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
+      <c r="N3" s="4" t="n"/>
+      <c r="O3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
@@ -1551,44 +1885,17 @@
       </c>
       <c r="K4" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N4" s="5" t="n"/>
       <c r="O4" s="5" t="n"/>
-      <c r="P4" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="R4" s="2" t="n"/>
-      <c r="S4" s="2" t="n"/>
-      <c r="T4" s="2" t="n"/>
-      <c r="U4" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V4" s="5" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="n">
@@ -1641,52 +1948,21 @@
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
+          <t>CARRIED_FORWARD</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="M5" s="6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260104.dat</t>
-        </is>
-      </c>
-      <c r="M5" s="6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N5" s="6" t="inlineStr">
-        <is>
-          <t>CARRIED_FORWARD</t>
-        </is>
-      </c>
-      <c r="O5" s="6" t="inlineStr">
-        <is>
-          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="P5" s="6" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q5" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="R5" s="2" t="n"/>
-      <c r="S5" s="2" t="n"/>
-      <c r="T5" s="2" t="n"/>
-      <c r="U5" s="6" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V5" s="6" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
+      <c r="N5" s="6" t="n"/>
+      <c r="O5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="n">
@@ -1739,44 +2015,17 @@
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>MISSING</t>
-        </is>
-      </c>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N6" s="5" t="n"/>
       <c r="O6" s="5" t="n"/>
-      <c r="P6" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q6" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="R6" s="2" t="n"/>
-      <c r="S6" s="2" t="n"/>
-      <c r="T6" s="2" t="n"/>
-      <c r="U6" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V6" s="5" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -1829,52 +2078,21 @@
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260106.dat</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t>NEW_FILE</t>
-        </is>
-      </c>
-      <c r="O7" s="4" t="inlineStr">
-        <is>
-          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="P7" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q7" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="R7" s="2" t="n"/>
-      <c r="S7" s="2" t="n"/>
-      <c r="T7" s="2" t="n"/>
-      <c r="U7" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V7" s="4" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
+      <c r="N7" s="4" t="n"/>
+      <c r="O7" s="4" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1927,52 +2145,21 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PARTCODR/ROPENS/1001/20260106.dat</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>NEW_FILE</t>
-        </is>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q8" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="R8" s="2" t="n"/>
-      <c r="S8" s="2" t="n"/>
-      <c r="T8" s="2" t="n"/>
-      <c r="U8" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V8" s="2" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
+      <c r="N8" s="2" t="n"/>
+      <c r="O8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -2025,52 +2212,21 @@
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PARTCODR/ROPENS/1002/20260109.dat</t>
-        </is>
-      </c>
-      <c r="M9" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t>NEW_FILE</t>
-        </is>
-      </c>
-      <c r="O9" s="4" t="inlineStr">
-        <is>
-          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="P9" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="Q9" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="R9" s="2" t="n"/>
-      <c r="S9" s="2" t="n"/>
-      <c r="T9" s="2" t="n"/>
-      <c r="U9" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V9" s="4" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
+      <c r="N9" s="4" t="n"/>
+      <c r="O9" s="4" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -2123,52 +2279,21 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PARTCODR/ROPENS/1003/20260106.dat</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>NEW_FILE</t>
-        </is>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q10" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="R10" s="2" t="n"/>
-      <c r="S10" s="2" t="n"/>
-      <c r="T10" s="2" t="n"/>
-      <c r="U10" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V10" s="2" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
+      <c r="N10" s="2" t="n"/>
+      <c r="O10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -2221,52 +2346,21 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>20260113_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PARTCODR/ROPENS/1001/20260113.dat</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>NEW_FILE</t>
-        </is>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>20260113_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q11" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="R11" s="2" t="n"/>
-      <c r="S11" s="2" t="n"/>
-      <c r="T11" s="2" t="n"/>
-      <c r="U11" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V11" s="2" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
+      <c r="N11" s="2" t="n"/>
+      <c r="O11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -2319,52 +2413,21 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>20260113_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PARTCODR/ROPENS/1002/20260113.dat</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N12" s="2" t="inlineStr">
-        <is>
-          <t>NEW_FILE</t>
-        </is>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>20260113_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q12" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="R12" s="2" t="n"/>
-      <c r="S12" s="2" t="n"/>
-      <c r="T12" s="2" t="n"/>
-      <c r="U12" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V12" s="2" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -2417,72 +2480,888 @@
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
+          <t>NEW_FILE</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="M13" s="4" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PARTCODR/ROPENS/1003/20260116.dat</t>
-        </is>
-      </c>
-      <c r="M13" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t>NEW_FILE</t>
-        </is>
-      </c>
-      <c r="O13" s="4" t="inlineStr">
-        <is>
-          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="P13" s="4" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="Q13" s="2" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="R13" s="2" t="inlineStr">
-        <is>
-          <t>mgarcia</t>
-        </is>
-      </c>
-      <c r="S13" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-14 13:00:00 (cleared 2026-01-16)</t>
-        </is>
-      </c>
-      <c r="T13" s="2" t="inlineStr">
-        <is>
-          <t>Corrected file approved Jan 16 - flag resolved</t>
-        </is>
-      </c>
-      <c r="U13" s="4" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="V13" s="4" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
+      <c r="N13" s="4" t="n"/>
+      <c r="O13" s="4" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V13"/>
+  <autoFilter ref="A1:O13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Detail_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>Req_ID</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>Btch_ID</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>Event_Ty</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>Received_File_Ref</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Batch_Closed_By</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Flagged_By</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>Flag_Rsn</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>Actor</t>
+        </is>
+      </c>
+      <c r="J1" s="3" t="inlineStr">
+        <is>
+          <t>Event_Dtts</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>FILE_RECEIVED</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260101.dat</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>BATCH_CLOSED</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>FILE_RECEIVED</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260102.dat</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="n"/>
+      <c r="G4" s="2" t="n"/>
+      <c r="H4" s="2" t="n"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>BATCH_CLOSED</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n"/>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="n"/>
+      <c r="H5" s="2" t="n"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>20260103_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BATCH_CLOSED</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>FILE_LOADED_NOT_PROMOTED</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260104.dat</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>BATCH_CLOSED</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>20260105_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>BATCH_CLOSED</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n"/>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>FILE_RECEIVED</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PROGAUDIT/ODAG1/2001/20260106.dat</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>BATCH_CLOSED</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n"/>
+      <c r="H11" s="2" t="n"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>FILE_RECEIVED</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1001/20260106.dat</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>BATCH_CLOSED</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>LATE_ARRIVAL</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1002/20260109.dat</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="n"/>
+      <c r="H14" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>BATCH_CLOSED</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>FILE_RECEIVED</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1003/20260106.dat</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="n"/>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>BATCH_CLOSED</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>20260113_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>FILE_RECEIVED</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1001/20260113.dat</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>20260113_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>BATCH_CLOSED</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>20260113_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>FILE_RECEIVED</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1002/20260113.dat</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>20260113_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>BATCH_CLOSED</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>FILE_RECEIVED</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/PARTCODR/ROPENS/1003/20260116.dat</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>BATCH_CLOSED</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>SYSTEM</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>CORRECTION_FLAGGED</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>mgarcia</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>1003's Jan 12 file passed rules validation but manual review found incorrect data - requesting corrected file from vendor</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>mgarcia</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-14 13:00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>CORRECTION_FLAG_CLEARED</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Corrected file approved</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>jsmith</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-16 10:15:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J25"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2963,7 +3842,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3245,423 +4124,4 @@
   <autoFilter ref="A1:M4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Event_ID</t>
-        </is>
-      </c>
-      <c r="B1" s="3" t="inlineStr">
-        <is>
-          <t>Btch_ID</t>
-        </is>
-      </c>
-      <c r="C1" s="3" t="inlineStr">
-        <is>
-          <t>Event_Ctgy</t>
-        </is>
-      </c>
-      <c r="D1" s="3" t="inlineStr">
-        <is>
-          <t>Event_Ty</t>
-        </is>
-      </c>
-      <c r="E1" s="3" t="inlineStr">
-        <is>
-          <t>Sevrty</t>
-        </is>
-      </c>
-      <c r="F1" s="3" t="inlineStr">
-        <is>
-          <t>Actor</t>
-        </is>
-      </c>
-      <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>Event_Dtts</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>20260103_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>EXCEPTION</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>SOURCE_MISSING_AT_COMBINE</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-03 20:00:00</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>FDR 2001 no approved anchor available for Jan 3 (candidate still PENDING_REVIEW at run time)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>AUDIT</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>FILE_RECEIVED_ANCHOR_ACTIVE</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-04 06:00:00</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>File received and loaded for Jan 4 but NOT used for the extract - approved anchor (Day 2 batch) still active and valid through 2026-01-31</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>AUDIT</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>CARRY_FORWARD_ANCHOR_REVOKED</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>mgarcia</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-05 07:30:00</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Anchor (Day 2 batch) revoked - data quality issue found; grouping now open for a new anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>20260106_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>EXCEPTION</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>SOURCE_MISSING_AT_COMBINE</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-06 20:00:00</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>FDR 1002 file not received for Jan 5 by SLA cutoff - extract closed PARTIAL, [1001,1003] only</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>EXCEPTION</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>DUPLICATE_FILE_IGNORED</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-07 08:00:00</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Duplicate resend of 1001's Jan 5 file - checksum matched, quarantined, no CRC/Override write</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>EXCEPTION</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>UNRECOGNIZED_SOURCE</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>SYSTEM</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-07 08:05:00</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>File from src=9999 not in ComplianceDataSetSourceXwalk - quarantined, no CRC/Override write</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>AUDIT</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>LATE_ARRIVAL_REOPEN_APPROVED</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>jsmith</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-09 11:40:00</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Late file accepted for 1002, Jan 5 (3 days late) - CRC row and extract reopened/regenerated/reclosed</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>20260113_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>EXCEPTION</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>DATA_QUALITY_ISSUE_FLAGGED</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>WARNING</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>mgarcia</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-14 13:00:00</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>1003's Jan 12 file passed rules validation but was found to contain incorrect data on manual review - corrected file requested from vendor</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>20260116_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>AUDIT</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>CORRECTION_REOPEN_APPROVED</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>INFO</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>jsmith</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>2026-01-16 10:15:00</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Corrected file accepted for 1003, Jan 12 - CRC row and extract reopened/regenerated/reclosed</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:H10"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add standalone interactive stepper (no chat-host dependency); rename project/source identifiers to Universe(210/Facets) and ODR(50/Qnxt,51/MHK,64/ESI) throughout mock data and docs
</commit_message>
<xml_diff>
--- a/mock-data/cms_compliance_framework_tables.xlsx
+++ b/mock-data/cms_compliance_framework_tables.xlsx
@@ -37,7 +37,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -60,14 +60,8 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="00666666"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -110,12 +104,6 @@
         <bgColor rgb="00EAD1F2"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFE699"/>
-        <bgColor rgb="00FFE699"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -143,29 +131,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -540,17 +525,17 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tab Name</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Contents</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Data Rows</t>
         </is>
@@ -568,7 +553,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -579,7 +564,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Source master (schema reference)</t>
+          <t>Source master - 210/Facets (Universe), 50/Qnxt, 51/MHK, 64/ESI (ODR)</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -594,7 +579,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Run type master - CMS (fixed reporting period) and DAILY (single day) used in the examples</t>
+          <t>Run type master - CMS (fixed reporting period) and DAILY (single day)</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -609,7 +594,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Carry-forward eligibility + config, per source/run type (schema reference)</t>
+          <t>Carry-forward eligibility + config, per source/run type</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -624,7 +609,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The one table a human writes to directly - data-quality flags and other genuinely business-initiated asks</t>
+          <t>The one table a human writes to directly - data-quality flags and other business-initiated asks</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -639,7 +624,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>CRC - continuous daily batches for Part C ODR (Jan 5-14, 3 FDRs); Btch_ID is Req_Dt_Key-based and NEVER changes on reopen</t>
+          <t>CRC - UNIVERSE/ODAG1 (Facets) + ODR/ROPENS (Qnxt, MHK, ESI) continuous daily Jan 5-14. Btch_ID is Req_Dt_Key-based, never changes on reopen</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -669,7 +654,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Sparse gate - Created_By_Ty/Current_State_By_Ty show system vs human. Btch_ID stable across reopen</t>
+          <t>Sparse gate - Created_By_Ty/Current_State_By_Ty show system vs human</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -684,7 +669,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>One row PER DAY - shows PARTIAL/COMPLETE and reopen/regenerate for every day in the Part C ODR range</t>
+          <t>One row PER DAY - PARTIAL/COMPLETE and reopen/regenerate across the ODR daily range</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -699,7 +684,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Append-only narrative log - data-quality flags, reopen approvals, upstream-rejected files</t>
+          <t>Append-only narrative log</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -736,67 +721,67 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Extract_ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Project_Cd</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Table_Nm</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Req_Dt_Key</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Extract_Stat</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Included_Src_Cds</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Missing_Src_Cds</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Extract_Generated_Dtts</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Extract_Close_Ind</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Extract_Closed_By</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>Reopen_Ind</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>Reopened_By</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>Reopen_Rsn</t>
         </is>
@@ -808,7 +793,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>PROGAUDIT</t>
+          <t>UNIVERSE</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -828,7 +813,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>[2001]</t>
+          <t>[210]</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -860,67 +845,67 @@
       <c r="M2" s="2" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="n">
+      <c r="A3" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>PARTCODR</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="B3" s="10" t="inlineStr">
+        <is>
+          <t>ODR</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t>ROPENS</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="10" t="inlineStr">
         <is>
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="10" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>[1001,1002,1003]</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>[50,51,64]</t>
+        </is>
+      </c>
+      <c r="G3" s="10" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="H3" s="10" t="inlineStr">
         <is>
           <t>2026-01-09 12:05:00</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" s="10" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="J3" s="10" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="K3" s="10" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="L3" s="10" t="inlineStr">
         <is>
           <t>jsmith</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
-        <is>
-          <t>1002 late-arrival approved Jan 9 - regenerated COMPLETE</t>
+      <c r="M3" s="10" t="inlineStr">
+        <is>
+          <t>MHK late-arrival approved Jan 9 - regenerated COMPLETE</t>
         </is>
       </c>
     </row>
@@ -930,7 +915,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -950,7 +935,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>[1001,1002,1003]</t>
+          <t>[50,51,64]</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -987,7 +972,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -1007,7 +992,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>[1001,1002,1003]</t>
+          <t>[50,51,64]</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1044,7 +1029,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -1064,7 +1049,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>[1001,1002,1003]</t>
+          <t>[50,51,64]</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1101,7 +1086,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1121,7 +1106,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>[1001,1002,1003]</t>
+          <t>[50,51,64]</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1153,67 +1138,67 @@
       <c r="M7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="n">
+      <c r="A8" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>PARTCODR</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>ODR</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>ROPENS</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="10" t="inlineStr">
         <is>
           <t>2026-01-10</t>
         </is>
       </c>
-      <c r="E8" s="5" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>COMPLETE</t>
         </is>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>[1001,1002,1003]</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>[50,51,64]</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="H8" s="5" t="inlineStr">
+      <c r="H8" s="10" t="inlineStr">
         <is>
           <t>2026-01-14 12:10:00</t>
         </is>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" s="10" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="J8" s="5" t="inlineStr">
+      <c r="J8" s="10" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="K8" s="10" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr">
+      <c r="L8" s="10" t="inlineStr">
         <is>
           <t>jsmith</t>
         </is>
       </c>
-      <c r="M8" s="5" t="inlineStr">
-        <is>
-          <t>1003 correction approved Jan 14 - regenerated with corrected batch</t>
+      <c r="M8" s="10" t="inlineStr">
+        <is>
+          <t>ESI correction approved Jan 14 - regenerated with corrected batch</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1208,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1243,7 +1228,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>[1001,1002,1003]</t>
+          <t>[50,51,64]</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -1280,7 +1265,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1300,7 +1285,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>[1001,1002,1003]</t>
+          <t>[50,51,64]</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -1337,7 +1322,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1357,7 +1342,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>[1001,1002,1003]</t>
+          <t>[50,51,64]</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1394,7 +1379,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1414,7 +1399,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>[1001,1002,1003]</t>
+          <t>[50,51,64]</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1461,7 +1446,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -1471,42 +1456,42 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Event_ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Btch_ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Event_Ctgy</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Event_Ty</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Sevrty</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Actor</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Event_Dtts</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -1518,7 +1503,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>20260103_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+          <t>20260103_UNIVERSE_ODAG1_210_CMS_2026_1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1548,7 +1533,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>FDR 2001 no approved anchor available for Jan 3 (candidate still PENDING_REVIEW at run time)</t>
+          <t>Facets no approved anchor available for Jan 3 (candidate still PENDING_REVIEW at run time)</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1543,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+          <t>20260106_UNIVERSE_ODAG1_210_CMS_2026_1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1598,7 +1583,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>20260105_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260105_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -1628,7 +1613,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>FDR 1002 file not received for Jan 5 by SLA cutoff - extract closed PARTIAL, [1001,1003] only</t>
+          <t>MHK file not received for Jan 5 by SLA cutoff - extract closed PARTIAL, [50,64] only</t>
         </is>
       </c>
     </row>
@@ -1664,7 +1649,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Duplicate resend of 1001's Jan 6 file - checksum matched, quarantined, no CRC/Override write</t>
+          <t>Duplicate resend of Qnxt's Jan 6 file - checksum matched, quarantined, no CRC/Override write</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1685,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>File from src=9999 not in ComplianceDataSetSourceXwalk - quarantined, no CRC/Override write</t>
+          <t>File from an unrecognized source code not in ComplianceDataSetSourceXwalk - quarantined, no CRC/Override write</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1695,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>20260105_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260105_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1740,7 +1725,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Late file accepted for 1002, Jan 5 (4 days late) - CRC row and extract reopened/regenerated/reclosed</t>
+          <t>Late file accepted for MHK, Jan 5 (4 days late) - CRC row and extract reopened/regenerated/reclosed</t>
         </is>
       </c>
     </row>
@@ -1750,7 +1735,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1780,7 +1765,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>1003's Jan 10 file passed rules validation but was found to contain incorrect data on manual review</t>
+          <t>ESI's Jan 10 file passed rules validation but was found to contain incorrect data on manual review</t>
         </is>
       </c>
     </row>
@@ -1790,7 +1775,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1820,7 +1805,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Corrected file accepted for 1003, Jan 10 - CRC row and extract reopened/regenerated/reclosed</t>
+          <t>Corrected file accepted for ESI, Jan 10 - CRC row and extract reopened/regenerated/reclosed</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1845,84 +1830,74 @@
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Color / Column</t>
         </is>
       </c>
-      <c r="B1" s="8" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
-      <c r="C1" s="8" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Where it appears</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
-      <c r="A2" s="9" t="inlineStr">
+    <row r="2" ht="55" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="B2" s="10" t="inlineStr">
-        <is>
-          <t>System-written - no human involved in this specific event/state</t>
-        </is>
-      </c>
-      <c r="C2" s="10" t="inlineStr">
-        <is>
-          <t>ComplianceRequestFileDetail.Entry_Ty; ComplianceBatchOverride.Created_By_Ty (always AUTO) and Current_State_By_Ty while PENDING_REVIEW</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>System-written - no human involved</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>ComplianceRequestFileDetail.Entry_Ty; Override.Created_By_Ty (always AUTO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="55" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>A human wrote or changed this - approval, revocation, or a business flag</t>
-        </is>
-      </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>ComplianceRequestFileDetail.Entry_Ty (CORRECTION_FLAGGED/CLEARED); ComplianceBatchOverride.Current_State_By_Ty when APPROVED or REVOKED</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>A human wrote or changed this</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Entry_Ty (flag events); Override.Current_State_By_Ty when APPROVED/REVOKED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="55" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
         <is>
           <t>Y (amber)</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
-        <is>
-          <t>This CRC row was updated in place after its original creation - a reopen touched it. Btch_ID is Req_Dt_Key-based and stays the SAME value even after this update (see framework-master.md section 5)</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>CRC row updated in place after creation. Btch_ID (Req_Dt_Key-based) stays the SAME value even after this update</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>ComplianceRequestControl.Row_Updated_Since_Creation_Ind</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Note: Part C ODR (ComplianceRequestControl rows for PARTCODR/ROPENS) now spans continuous daily batches Jan 5-14 for all 3 FDRs - 30 routine rows plus the 2 highlighted (orange fill) rows that were reopened. This replaces the earlier 2-isolated-date version.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A6:C6"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1937,28 +1912,28 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Src_Cd</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Src_Nm</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Src_Ty</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Active_Ind</t>
         </is>
@@ -1967,12 +1942,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2001</t>
+          <t>210</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Vendor FDR 2001</t>
+          <t>Facets</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -1989,12 +1964,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Vendor FDR 1001</t>
+          <t>Qnxt</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -2011,12 +1986,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Vendor FDR 1002</t>
+          <t>MHK</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -2033,12 +2008,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Vendor FDR 1003</t>
+          <t>ESI</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -2073,17 +2048,17 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Run_Ty</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Run_Ty_Desc</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>SLA_Days</t>
         </is>
@@ -2143,32 +2118,32 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Project_Cd</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Table_Nm</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Src_Cd</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Run_Ty</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Cmplnc_Vrsn</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Carry_Fwd_Elig_Ind</t>
         </is>
@@ -2177,7 +2152,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PROGAUDIT</t>
+          <t>UNIVERSE</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -2187,7 +2162,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2001</t>
+          <t>210</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -2209,7 +2184,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -2219,7 +2194,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>50</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -2241,7 +2216,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -2251,7 +2226,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>51</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -2273,7 +2248,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -2283,7 +2258,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -2331,57 +2306,57 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Intake_ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Project_Cd</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Table_Nm</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Src_Cd</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Req_Dt_Key</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Req_Ty</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Requested_By</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Requested_Dtts</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Rsn</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Processed_Ind</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>Processed_Dtts</t>
         </is>
@@ -2395,7 +2370,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -2405,7 +2380,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -2430,7 +2405,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>1003's Jan 10 file passed rules validation but manual review found incorrect data - requesting corrected file from vendor</t>
+          <t>ESI's Jan 10 file passed rules validation but manual review found incorrect data - requesting corrected file from vendor</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -2467,493 +2442,493 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
-    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
     <col width="32" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Req_ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Project_Cd</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Table_Nm</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Src_Cd</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Run_Ty</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Req_Dt_Key</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Rpt_Start_Dt_Key</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Rpt_End_Dt_Key</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Btch_ID</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Req_Stat</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>Resolution_Ty</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>Used_Btch_ID</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>Batch_Close_Ind</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="7" t="inlineStr">
         <is>
           <t>Row_Updated_Since_Creation_Ind</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>PROGAUDIT</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>UNIVERSE</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
         <is>
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
         <is>
           <t>CMS</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="8" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="8" t="inlineStr">
         <is>
           <t>2026-01-31</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>20260101_UNIVERSE_ODAG1_210_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
         <is>
           <t>RULES_PASSED</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="8" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
-        <is>
-          <t>20260101_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="L2" s="8" t="inlineStr">
+        <is>
+          <t>20260101_UNIVERSE_ODAG1_210_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="M2" s="8" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="N2" s="8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>PROGAUDIT</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>UNIVERSE</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
         <is>
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
         <is>
           <t>CMS</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" s="8" t="inlineStr">
         <is>
           <t>2026-01-02</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="H3" s="8" t="inlineStr">
         <is>
           <t>2026-01-31</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>20260102_UNIVERSE_ODAG1_210_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
         <is>
           <t>RULES_PASSED</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" s="8" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>20260102_UNIVERSE_ODAG1_210_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="N3" s="8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="n">
+      <c r="A4" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>PROGAUDIT</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>UNIVERSE</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t>CMS</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>2026-01-03</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="9" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="9" t="inlineStr">
         <is>
           <t>2026-01-31</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>20260103_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>20260103_UNIVERSE_ODAG1_210_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>DATA_NOT_PROVIDED</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="K4" s="9" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="L4" s="4" t="n"/>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="L4" s="9" t="n"/>
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="N4" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="n">
+      <c r="A5" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>PROGAUDIT</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>UNIVERSE</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>CMS</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t>2026-01-04</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="10" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>2026-01-31</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>20260104_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>20260104_UNIVERSE_ODAG1_210_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
         <is>
           <t>EXTRACTED</t>
         </is>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="K5" s="10" t="inlineStr">
         <is>
           <t>CARRIED_FORWARD</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>20260102_UNIVERSE_ODAG1_210_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr">
+      <c r="N5" s="10" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>PROGAUDIT</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>UNIVERSE</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>CMS</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="9" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="9" t="inlineStr">
         <is>
           <t>2026-01-31</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>20260105_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="I6" s="9" t="inlineStr">
+        <is>
+          <t>20260105_UNIVERSE_ODAG1_210_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J6" s="9" t="inlineStr">
         <is>
           <t>DATA_NOT_PROVIDED</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K6" s="9" t="inlineStr">
         <is>
           <t>MISSING</t>
         </is>
       </c>
-      <c r="L6" s="4" t="n"/>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="L6" s="9" t="n"/>
+      <c r="M6" s="9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="N6" s="9" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>PROGAUDIT</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>UNIVERSE</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
         <is>
           <t>ODAG1</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>2001</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>210</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>CMS</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="8" t="inlineStr">
         <is>
           <t>2026-01-06</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="8" t="inlineStr">
         <is>
           <t>2026-01-01</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H7" s="8" t="inlineStr">
         <is>
           <t>2026-01-31</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
-        <is>
-          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>20260106_UNIVERSE_ODAG1_210_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
         <is>
           <t>RULES_PASSED</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" s="8" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
-        <is>
-          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
-        </is>
-      </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>20260106_UNIVERSE_ODAG1_210_CMS_2026_1</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="N7" s="3" t="inlineStr">
+      <c r="N7" s="8" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2965,7 +2940,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -2975,7 +2950,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -3000,7 +2975,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>20260105_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260105_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
@@ -3015,7 +2990,7 @@
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>20260105_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260105_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
@@ -3030,70 +3005,70 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>PARTCODR</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>ODR</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
         <is>
           <t>ROPENS</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>1002</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>DAILY</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="8" t="inlineStr">
         <is>
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
         <is>
           <t>2026-01-05</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>20260105_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="J9" s="3" t="inlineStr">
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>20260105_ODR_ROPENS_51_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>EXTRACTED</t>
         </is>
       </c>
-      <c r="K9" s="3" t="inlineStr">
+      <c r="K9" s="8" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
-          <t>20260105_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="M9" s="3" t="inlineStr">
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>20260105_ODR_ROPENS_51_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="N9" s="3" t="inlineStr">
+      <c r="N9" s="8" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -3105,7 +3080,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -3115,7 +3090,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -3140,7 +3115,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>20260105_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260105_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -3155,7 +3130,7 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>20260105_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260105_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
@@ -3175,7 +3150,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -3185,7 +3160,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -3210,7 +3185,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260106_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -3225,7 +3200,7 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260106_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
@@ -3245,7 +3220,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -3255,7 +3230,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>51</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -3280,7 +3255,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>20260106_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260106_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -3295,7 +3270,7 @@
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>20260106_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260106_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
@@ -3315,7 +3290,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -3325,7 +3300,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
@@ -3350,7 +3325,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260106_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -3365,7 +3340,7 @@
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>20260106_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260106_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -3385,7 +3360,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -3395,7 +3370,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -3420,7 +3395,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>20260107_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260107_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -3435,7 +3410,7 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>20260107_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260107_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -3455,7 +3430,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -3465,7 +3440,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>51</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -3490,7 +3465,7 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>20260107_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260107_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
@@ -3505,7 +3480,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>20260107_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260107_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -3525,7 +3500,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -3535,7 +3510,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -3560,7 +3535,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>20260107_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260107_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
@@ -3575,7 +3550,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>20260107_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260107_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -3595,7 +3570,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -3605,7 +3580,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -3630,7 +3605,7 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>20260108_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260108_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
@@ -3645,7 +3620,7 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>20260108_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260108_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M17" s="2" t="inlineStr">
@@ -3665,7 +3640,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -3675,7 +3650,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>51</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -3700,7 +3675,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>20260108_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260108_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -3715,7 +3690,7 @@
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>20260108_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260108_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -3735,7 +3710,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -3745,7 +3720,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -3770,7 +3745,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260108_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -3785,7 +3760,7 @@
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>20260108_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260108_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M19" s="2" t="inlineStr">
@@ -3805,7 +3780,7 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -3815,7 +3790,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -3840,7 +3815,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>20260109_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260109_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -3855,7 +3830,7 @@
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>20260109_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260109_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M20" s="2" t="inlineStr">
@@ -3875,7 +3850,7 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -3885,7 +3860,7 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>51</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -3910,7 +3885,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260109_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -3925,7 +3900,7 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>20260109_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260109_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M21" s="2" t="inlineStr">
@@ -3945,7 +3920,7 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -3955,7 +3930,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -3980,7 +3955,7 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>20260109_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260109_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -3995,7 +3970,7 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>20260109_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260109_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M22" s="2" t="inlineStr">
@@ -4015,7 +3990,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -4025,7 +4000,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -4050,7 +4025,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>20260110_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260110_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -4065,7 +4040,7 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>20260110_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260110_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M23" s="2" t="inlineStr">
@@ -4085,7 +4060,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -4095,7 +4070,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>51</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -4120,7 +4095,7 @@
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>20260110_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260110_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -4135,7 +4110,7 @@
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>20260110_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260110_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M24" s="2" t="inlineStr">
@@ -4150,70 +4125,70 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n">
+      <c r="A25" s="8" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>PARTCODR</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>ODR</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
         <is>
           <t>ROPENS</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
-        <is>
-          <t>1003</t>
-        </is>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>DAILY</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F25" s="8" t="inlineStr">
         <is>
           <t>2026-01-10</t>
         </is>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G25" s="8" t="inlineStr">
         <is>
           <t>2026-01-10</t>
         </is>
       </c>
-      <c r="H25" s="3" t="inlineStr">
+      <c r="H25" s="8" t="inlineStr">
         <is>
           <t>2026-01-10</t>
         </is>
       </c>
-      <c r="I25" s="3" t="inlineStr">
-        <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="J25" s="3" t="inlineStr">
+      <c r="I25" s="8" t="inlineStr">
+        <is>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="J25" s="8" t="inlineStr">
         <is>
           <t>EXTRACTED</t>
         </is>
       </c>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="K25" s="8" t="inlineStr">
         <is>
           <t>NEW_FILE</t>
         </is>
       </c>
-      <c r="L25" s="3" t="inlineStr">
-        <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="M25" s="3" t="inlineStr">
+      <c r="L25" s="8" t="inlineStr">
+        <is>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="M25" s="8" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="N25" s="3" t="inlineStr">
+      <c r="N25" s="8" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -4225,7 +4200,7 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -4235,7 +4210,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -4260,7 +4235,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>20260111_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260111_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -4275,7 +4250,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>20260111_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260111_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -4295,7 +4270,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -4305,7 +4280,7 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>51</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
@@ -4330,7 +4305,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>20260111_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260111_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -4345,7 +4320,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>20260111_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260111_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M27" s="2" t="inlineStr">
@@ -4365,7 +4340,7 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -4375,7 +4350,7 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -4400,7 +4375,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>20260111_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260111_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -4415,7 +4390,7 @@
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>20260111_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260111_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M28" s="2" t="inlineStr">
@@ -4435,7 +4410,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -4445,7 +4420,7 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -4470,7 +4445,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>20260112_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260112_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -4485,7 +4460,7 @@
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>20260112_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260112_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M29" s="2" t="inlineStr">
@@ -4505,7 +4480,7 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -4515,7 +4490,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>51</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -4540,7 +4515,7 @@
       </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>20260112_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260112_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
@@ -4555,7 +4530,7 @@
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>20260112_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260112_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M30" s="2" t="inlineStr">
@@ -4575,7 +4550,7 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -4585,7 +4560,7 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -4610,7 +4585,7 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>20260112_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260112_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -4625,7 +4600,7 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>20260112_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260112_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
@@ -4645,7 +4620,7 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -4655,7 +4630,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -4680,7 +4655,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>20260113_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260113_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -4695,7 +4670,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>20260113_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260113_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
@@ -4715,7 +4690,7 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -4725,7 +4700,7 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>51</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -4750,7 +4725,7 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>20260113_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260113_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -4765,7 +4740,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>20260113_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260113_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M33" s="2" t="inlineStr">
@@ -4785,7 +4760,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -4795,7 +4770,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -4820,7 +4795,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>20260113_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260113_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -4835,7 +4810,7 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>20260113_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260113_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M34" s="2" t="inlineStr">
@@ -4855,7 +4830,7 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -4865,7 +4840,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>1001</t>
+          <t>50</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -4890,7 +4865,7 @@
       </c>
       <c r="I35" s="2" t="inlineStr">
         <is>
-          <t>20260114_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260114_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -4905,7 +4880,7 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>20260114_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
+          <t>20260114_ODR_ROPENS_50_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
@@ -4925,7 +4900,7 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -4935,7 +4910,7 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>51</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
@@ -4960,7 +4935,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>20260114_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260114_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -4975,7 +4950,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>20260114_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260114_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M36" s="2" t="inlineStr">
@@ -4995,7 +4970,7 @@
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -5005,7 +4980,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -5030,7 +5005,7 @@
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>20260114_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260114_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -5045,7 +5020,7 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>20260114_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260114_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
@@ -5076,7 +5051,7 @@
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="46" customWidth="1" min="6" max="6"/>
@@ -5088,508 +5063,508 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Detail_ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Req_ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Btch_ID</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Event_Ty</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Entry_Ty</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Received_File_Ref</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Batch_Closed_By</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Flagged_By</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Flag_Rsn</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Actor</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>Event_Dtts</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="n">
+      <c r="A2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="n">
+      <c r="B2" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
+        <is>
+          <t>20260106_ODR_ROPENS_50_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D2" s="11" t="inlineStr">
         <is>
           <t>FILE_RECEIVED</t>
         </is>
       </c>
-      <c r="E2" s="6" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="F2" s="6" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PARTCODR/ROPENS/1001/20260106.dat</t>
-        </is>
-      </c>
-      <c r="G2" s="6" t="n"/>
-      <c r="H2" s="6" t="n"/>
-      <c r="I2" s="6" t="n"/>
-      <c r="J2" s="6" t="inlineStr">
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/ODR/ROPENS/50/20260106.dat</t>
+        </is>
+      </c>
+      <c r="G2" s="11" t="n"/>
+      <c r="H2" s="11" t="n"/>
+      <c r="I2" s="11" t="n"/>
+      <c r="J2" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="K2" s="6" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>2026-01-06 06:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B3" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>20260106_PARTCODR_ROPENS_1001_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>20260106_ODR_ROPENS_50_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
         <is>
           <t>BATCH_CLOSED</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="inlineStr">
+      <c r="F3" s="11" t="n"/>
+      <c r="G3" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="H3" s="11" t="n"/>
+      <c r="I3" s="11" t="n"/>
+      <c r="J3" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="K3" s="11" t="inlineStr">
         <is>
           <t>2026-01-06 20:00:00</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n">
+      <c r="A4" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>20260105_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
+        <is>
+          <t>20260105_ODR_ROPENS_51_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D4" s="11" t="inlineStr">
         <is>
           <t>BATCH_CLOSED</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="F4" s="11" t="n"/>
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="inlineStr">
+      <c r="H4" s="11" t="n"/>
+      <c r="I4" s="11" t="n"/>
+      <c r="J4" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="K4" s="6" t="inlineStr">
+      <c r="K4" s="11" t="inlineStr">
         <is>
           <t>2026-01-05 20:00:00</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>20260105_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>20260105_ODR_ROPENS_51_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>LATE_ARRIVAL</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PARTCODR/ROPENS/1002/20260109-late.dat</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
-      <c r="J5" s="6" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/ODR/ROPENS/51/20260109-late.dat</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="n"/>
+      <c r="H5" s="11" t="n"/>
+      <c r="I5" s="11" t="n"/>
+      <c r="J5" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="K5" s="11" t="inlineStr">
         <is>
           <t>2026-01-09 08:30:00</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n">
+      <c r="A6" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>20260105_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>20260105_ODR_ROPENS_51_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>BATCH_CLOSED</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="F6" s="11" t="n"/>
+      <c r="G6" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
-      <c r="J6" s="6" t="inlineStr">
+      <c r="H6" s="11" t="n"/>
+      <c r="I6" s="11" t="n"/>
+      <c r="J6" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>2026-01-09 12:05:00</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n">
+      <c r="A7" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>FILE_RECEIVED</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PARTCODR/ROPENS/1003/20260110.dat</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/ODR/ROPENS/64/20260110.dat</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="11" t="n"/>
+      <c r="I7" s="11" t="n"/>
+      <c r="J7" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>2026-01-10 06:00:00</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n">
+      <c r="A8" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>BATCH_CLOSED</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="6" t="inlineStr">
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="6" t="n"/>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="H8" s="11" t="n"/>
+      <c r="I8" s="11" t="n"/>
+      <c r="J8" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>2026-01-10 20:00:00</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="n">
+      <c r="A9" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="n">
+      <c r="B9" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>CORRECTION_FLAGGED</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="12" t="inlineStr">
         <is>
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="12" t="inlineStr">
         <is>
           <t>mgarcia</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
-        <is>
-          <t>1003's Jan 10 file passed rules validation but manual review found incorrect data</t>
-        </is>
-      </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>ESI's Jan 10 file passed rules validation but manual review found incorrect data</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
         <is>
           <t>mgarcia</t>
         </is>
       </c>
-      <c r="K9" s="7" t="inlineStr">
+      <c r="K9" s="12" t="inlineStr">
         <is>
           <t>2026-01-12 13:00:00</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n">
+      <c r="A10" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>FILE_RECEIVED</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
-        <is>
-          <t>s3://cms-inbound/PARTCODR/ROPENS/1003/20260114-corrected.dat</t>
-        </is>
-      </c>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>s3://cms-inbound/ODR/ROPENS/64/20260114-corrected.dat</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="11" t="n"/>
+      <c r="I10" s="11" t="n"/>
+      <c r="J10" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>2026-01-14 09:10:00</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n">
+      <c r="A11" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="7" t="n">
+      <c r="B11" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
         <is>
           <t>CORRECTION_FLAG_CLEARED</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="12" t="inlineStr">
         <is>
           <t>MANUAL</t>
         </is>
       </c>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="inlineStr">
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="12" t="n"/>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="12" t="inlineStr">
         <is>
           <t>jsmith</t>
         </is>
       </c>
-      <c r="K11" s="7" t="inlineStr">
+      <c r="K11" s="12" t="inlineStr">
         <is>
           <t>2026-01-14 10:15:00</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n">
+      <c r="A12" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="11" t="n">
         <v>24</v>
       </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>BATCH_CLOSED</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>AUTO</t>
         </is>
       </c>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="6" t="n"/>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="H12" s="11" t="n"/>
+      <c r="I12" s="11" t="n"/>
+      <c r="J12" s="11" t="inlineStr">
         <is>
           <t>SYSTEM</t>
         </is>
       </c>
-      <c r="K12" s="6" t="inlineStr">
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>2026-01-14 12:10:00</t>
         </is>
@@ -5618,10 +5593,10 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
-    <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="37" customWidth="1" min="12" max="12"/>
     <col width="21" customWidth="1" min="13" max="13"/>
     <col width="15" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
@@ -5636,117 +5611,117 @@
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>Ovrd_ID</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Req_ID</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Project_Cd</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Table_Nm</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="7" t="inlineStr">
         <is>
           <t>Src_Cd</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Run_Ty</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Rpt_Start_Dt_Key</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Rpt_End_Dt_Key</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Btch_ID</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Used_Btch_ID</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>Override_Ty</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>Prior_Btch_ID</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>Prior_Resolution_Ty</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="7" t="inlineStr">
         <is>
           <t>Created_By_Ty</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="7" t="inlineStr">
         <is>
           <t>Apprvl_Stat</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="7" t="inlineStr">
         <is>
           <t>Current_State_By_Ty</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" s="7" t="inlineStr">
         <is>
           <t>Apprvd_By</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" s="7" t="inlineStr">
         <is>
           <t>Apprvd_Dtts</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" s="7" t="inlineStr">
         <is>
           <t>Reuse_Valid_Thru_Dt_Key</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" s="7" t="inlineStr">
         <is>
           <t>Revoked_By</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" s="7" t="inlineStr">
         <is>
           <t>Revoked_Dtts</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" s="7" t="inlineStr">
         <is>
           <t>Revocation_Rsn</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" s="7" t="inlineStr">
         <is>
           <t>History</t>
         </is>
@@ -5761,7 +5736,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>PROGAUDIT</t>
+          <t>UNIVERSE</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -5771,7 +5746,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>2001</t>
+          <t>210</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -5791,12 +5766,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+          <t>20260102_UNIVERSE_ODAG1_210_CMS_2026_1</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>20260102_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+          <t>20260102_UNIVERSE_ODAG1_210_CMS_2026_1</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -5853,7 +5828,7 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>Day 1: row created, PENDING_REVIEW (candidate: Day 1 batch) | Day 2: candidate replaced with Day 2's batch, still PENDING_REVIEW | Day 2: UPDATE -&gt; APPROVED by jsmith, valid through 2026-01-31 | Day 3: UPDATE -&gt; REVOKED by mgarcia - data quality issue found</t>
+          <t>Day 1: row created, PENDING_REVIEW | Day 2: candidate replaced, still PENDING_REVIEW | Day 2: UPDATE -&gt; APPROVED by jsmith, valid through 2026-01-31 | Day 3: UPDATE -&gt; REVOKED by mgarcia</t>
         </is>
       </c>
     </row>
@@ -5866,7 +5841,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>PROGAUDIT</t>
+          <t>UNIVERSE</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -5876,7 +5851,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>2001</t>
+          <t>210</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -5896,12 +5871,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+          <t>20260106_UNIVERSE_ODAG1_210_CMS_2026_1</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>20260106_PROGAUDIT_ODAG1_2001_CMS_2026_1</t>
+          <t>20260106_UNIVERSE_ODAG1_210_CMS_2026_1</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -5934,7 +5909,7 @@
       <c r="V3" s="2" t="n"/>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>Day 6: row created, PENDING_REVIEW (candidate: Day 6 batch) - grouping free again after Day 3 revoke</t>
+          <t>Day 6: row created, PENDING_REVIEW - grouping free again after Day 3 revoke</t>
         </is>
       </c>
     </row>
@@ -5947,7 +5922,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -5957,7 +5932,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>1002</t>
+          <t>51</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -5977,12 +5952,12 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>20260105_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260105_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>20260105_PARTCODR_ROPENS_1002_DAILY_2026_1</t>
+          <t>20260105_ODR_ROPENS_51_DAILY_2026_1</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
@@ -6027,7 +6002,7 @@
       <c r="V4" s="2" t="n"/>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>Jan 9: row created, PENDING_REVIEW (late file received for closed/missing Jan-5 batch, 4 days late) | Jan 9: UPDATE -&gt; APPROVED by jsmith</t>
+          <t>Jan 9: row created, PENDING_REVIEW (MHK's late file for Jan 5, 4 days late) | Jan 9: UPDATE -&gt; APPROVED by jsmith</t>
         </is>
       </c>
     </row>
@@ -6040,7 +6015,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>PARTCODR</t>
+          <t>ODR</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -6050,7 +6025,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>1003</t>
+          <t>64</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -6070,12 +6045,12 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -6085,7 +6060,7 @@
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>20260110_PARTCODR_ROPENS_1003_DAILY_2026_1</t>
+          <t>20260110_ODR_ROPENS_64_DAILY_2026_1</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -6124,7 +6099,7 @@
       <c r="V5" s="2" t="n"/>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>Jan 14: row created, PENDING_REVIEW (corrected file received for closed Jan-10 batch - data quality issue flagged Jan 12) | Jan 14: UPDATE -&gt; APPROVED by jsmith</t>
+          <t>Jan 14: row created, PENDING_REVIEW (ESI's corrected file for Jan 10 - flagged Jan 12) | Jan 14: UPDATE -&gt; APPROVED by jsmith</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rename stepper to latearrival.html; add reuse-carryforward.html companion for the Universe carry-forward reuse scenario; fix Override approve/revoke timestamps to match the Day3/Day5 narrative
</commit_message>
<xml_diff>
--- a/mock-data/cms_compliance_framework_tables.xlsx
+++ b/mock-data/cms_compliance_framework_tables.xlsx
@@ -1568,7 +1568,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>2026-01-03 07:30:00</t>
+          <t>2026-01-05 07:30:00</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -5803,7 +5803,7 @@
       </c>
       <c r="R2" s="2" t="inlineStr">
         <is>
-          <t>2026-01-02 09:00:00</t>
+          <t>2026-01-03 20:15:00</t>
         </is>
       </c>
       <c r="S2" s="2" t="inlineStr">
@@ -5818,7 +5818,7 @@
       </c>
       <c r="U2" s="2" t="inlineStr">
         <is>
-          <t>2026-01-03 07:30:00</t>
+          <t>2026-01-05 07:30:00</t>
         </is>
       </c>
       <c r="V2" s="2" t="inlineStr">
@@ -5828,7 +5828,7 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>Day 1: row created, PENDING_REVIEW | Day 2: candidate replaced, still PENDING_REVIEW | Day 2: UPDATE -&gt; APPROVED by jsmith, valid through 2026-01-31 | Day 3: UPDATE -&gt; REVOKED by mgarcia</t>
+          <t>Day 1: row created, PENDING_REVIEW (candidate: Day 1 batch) | Day 2: candidate replaced with Day 2's batch, still PENDING_REVIEW | Day 3: UPDATE -&gt; APPROVED by jsmith, valid through 2026-01-31 | Day 5: UPDATE -&gt; REVOKED by mgarcia - data quality issue found</t>
         </is>
       </c>
     </row>

</xml_diff>